<commit_message>
More one time using it
</commit_message>
<xml_diff>
--- a/src/main/resources/baseFiles/excel/Sheet.xlsx
+++ b/src/main/resources/baseFiles/excel/Sheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14540"/>
+    <workbookView windowWidth="24680" windowHeight="14540"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -58,9 +58,6 @@
   <si>
     <t>Firm</t>
   </si>
-  <si>
-    <t/>
-  </si>
 </sst>
 </file>
 
@@ -225,18 +222,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -557,7 +548,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -581,16 +572,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -599,93 +590,92 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1223,38 +1213,45 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="A2:J372">
+    <sortCondition ref="D2:D372"/>
+    <sortCondition ref="J2:J372"/>
+    <sortCondition ref="I2:I372"/>
+    <sortCondition ref="F2:F372"/>
+    <sortCondition ref="C2:C372"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Before changing the SiteUtils function filterlawyersinpage
</commit_message>
<xml_diff>
--- a/src/main/resources/baseFiles/excel/Sheet.xlsx
+++ b/src/main/resources/baseFiles/excel/Sheet.xlsx
@@ -1213,34 +1213,34 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
     </row>

</xml_diff>